<commit_message>
Capture Tier A contact emails from the ZoomInfo pass
The Tier A enrichment returned verified contact emails alongside the phone
numbers, but only the phones were persisted. Adds a ContactEmail column to
targets.csv (42 Tier A emails), fills the Verified Email column in
call-list.csv, and carries both into the master workbook.

Nelco Products is deliberately left blank: ZoomInfo returned an address on
the flextronics.com domain, which is already flagged for verification.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013nq1bUVgNscLtNebgo7tRL
</commit_message>
<xml_diff>
--- a/5PT-Master-Prospecting-Workbook.xlsx
+++ b/5PT-Master-Prospecting-Workbook.xlsx
@@ -690,7 +690,11 @@
       </c>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>ccastellano@cutterassociates.com</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Cindy Castellano (Chief Executive Officer)</t>
@@ -1440,7 +1444,11 @@
           <t>Chief Information Officer</t>
         </is>
       </c>
-      <c r="M9" s="2" t="n"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>mfederico@rfcu.com</t>
+        </is>
+      </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
           <t>Kristin VanBeek (Chief Executive Officer &amp; President)</t>
@@ -1554,7 +1562,11 @@
           <t>Director, Information Technology</t>
         </is>
       </c>
-      <c r="M10" s="2" t="n"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>darrell@uppababy.com</t>
+        </is>
+      </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
           <t>Bob Monahan (Chief Executive Officer &amp; Co-Founder)</t>
@@ -1770,7 +1782,11 @@
       </c>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n"/>
-      <c r="M12" s="2" t="n"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>sskorohod@briggsengineering.com</t>
+        </is>
+      </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
           <t>Sean Skorohod (Testing Services President &amp; Director)</t>
@@ -3072,7 +3088,11 @@
           <t>Senior Director, Information Technology</t>
         </is>
       </c>
-      <c r="M25" s="2" t="n"/>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>jamesc@zildjian.com</t>
+        </is>
+      </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
           <t>Thomas Young (Senior Vice President, Chief Financial Officer and Treasurer)</t>
@@ -3296,7 +3316,11 @@
           <t>It Help Desk Technician</t>
         </is>
       </c>
-      <c r="M27" s="4" t="n"/>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>slutz@nvna.org</t>
+        </is>
+      </c>
       <c r="N27" s="4" t="inlineStr">
         <is>
           <t>Bj Snow (Chief Human Resources Officer)</t>
@@ -3520,7 +3544,11 @@
           <t>Chief Information Officer</t>
         </is>
       </c>
-      <c r="M29" s="2" t="n"/>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>wayne@miniter.com</t>
+        </is>
+      </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
           <t>Julianne Gilpin (President &amp; Chief Executive Officer)</t>
@@ -3622,7 +3650,11 @@
       <c r="J30" s="4" t="n"/>
       <c r="K30" s="4" t="n"/>
       <c r="L30" s="4" t="n"/>
-      <c r="M30" s="4" t="n"/>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>danielle.jones@snowandjones.com</t>
+        </is>
+      </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
           <t>Danielle Jones (President)</t>
@@ -3728,7 +3760,11 @@
       </c>
       <c r="K31" s="2" t="n"/>
       <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="n"/>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>randallsteele@airxchange.com</t>
+        </is>
+      </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
           <t>Randall Steele (President &amp; Chief Executive Officer)</t>
@@ -5830,7 +5866,11 @@
           <t>Manager, Network</t>
         </is>
       </c>
-      <c r="M52" s="2" t="n"/>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>emoniz@cushingcenters.org</t>
+        </is>
+      </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
           <t>Gina Rosas (Chief Operating Officer)</t>
@@ -6626,7 +6666,11 @@
           <t>Director, Information Technology</t>
         </is>
       </c>
-      <c r="M60" s="4" t="n"/>
+      <c r="M60" s="4" t="inlineStr">
+        <is>
+          <t>aemma@palanders.com</t>
+        </is>
+      </c>
       <c r="N60" s="4" t="inlineStr">
         <is>
           <t>Joseph Durant (Chief Operating Officer)</t>
@@ -6740,7 +6784,11 @@
           <t>Manager, Information Technology</t>
         </is>
       </c>
-      <c r="M61" s="2" t="n"/>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>dmelo@buckleyonline.com</t>
+        </is>
+      </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
           <t>Robert Buckley (Founder)</t>
@@ -6854,7 +6902,11 @@
           <t>Chief Information Officer</t>
         </is>
       </c>
-      <c r="M62" s="2" t="n"/>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>lraasch@srcmedical.com</t>
+        </is>
+      </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
           <t>Roy Tinkham (President)</t>
@@ -6968,7 +7020,11 @@
           <t>System Administrator</t>
         </is>
       </c>
-      <c r="M63" s="2" t="n"/>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>daniel_mcclelland@hapcoincorporated.com</t>
+        </is>
+      </c>
       <c r="N63" s="2" t="inlineStr">
         <is>
           <t>Fred DeSimone (General Manager)</t>
@@ -7078,7 +7134,11 @@
           <t>IT Administrator</t>
         </is>
       </c>
-      <c r="M64" s="4" t="n"/>
+      <c r="M64" s="4" t="inlineStr">
+        <is>
+          <t>mphung@gemgravure.com</t>
+        </is>
+      </c>
       <c r="N64" s="4" t="inlineStr">
         <is>
           <t>Joseph Gemelli (Founder)</t>
@@ -7968,7 +8028,11 @@
           <t>Manager, Information Technology</t>
         </is>
       </c>
-      <c r="M73" s="2" t="n"/>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>jnoel@royalhealthgroup.com</t>
+        </is>
+      </c>
       <c r="N73" s="2" t="inlineStr">
         <is>
           <t>Pamela Jones (Chief Financial Officer)</t>
@@ -8180,7 +8244,11 @@
           <t>Information Technology Consultant</t>
         </is>
       </c>
-      <c r="M75" s="2" t="n"/>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>cgeer@thayerscale.com</t>
+        </is>
+      </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
           <t>Frank Hyer (Chairman &amp; Chief Executive Officer)</t>
@@ -9898,7 +9966,11 @@
       </c>
       <c r="K92" s="2" t="n"/>
       <c r="L92" s="2" t="n"/>
-      <c r="M92" s="2" t="n"/>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>pcleary@tkasphalt.com</t>
+        </is>
+      </c>
       <c r="N92" s="2" t="inlineStr">
         <is>
           <t>Peter Cleary (Chief Financial Officer)</t>
@@ -10000,7 +10072,11 @@
       <c r="J93" s="4" t="n"/>
       <c r="K93" s="4" t="n"/>
       <c r="L93" s="4" t="n"/>
-      <c r="M93" s="4" t="n"/>
+      <c r="M93" s="4" t="inlineStr">
+        <is>
+          <t>tmcmanus@cclco.com</t>
+        </is>
+      </c>
       <c r="N93" s="4" t="inlineStr">
         <is>
           <t>Thomas McManus (President)</t>
@@ -11172,7 +11248,11 @@
           <t>Vice President and Information Technology Operations Ma...</t>
         </is>
       </c>
-      <c r="M105" s="4" t="n"/>
+      <c r="M105" s="4" t="inlineStr">
+        <is>
+          <t>ltempesta@southshorebank.com</t>
+        </is>
+      </c>
       <c r="N105" s="4" t="inlineStr">
         <is>
           <t>James Dunphy (President &amp; Chief Executive Officer)</t>
@@ -11290,7 +11370,11 @@
           <t>Manager, Corporate Information Systems</t>
         </is>
       </c>
-      <c r="M106" s="2" t="n"/>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>kroche@electroswitch.com</t>
+        </is>
+      </c>
       <c r="N106" s="2" t="n"/>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -11400,7 +11484,11 @@
           <t>Vice President, Information Technology &amp; Officer</t>
         </is>
       </c>
-      <c r="M107" s="2" t="n"/>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>mruuska@coastalheritagebank.com</t>
+        </is>
+      </c>
       <c r="N107" s="2" t="inlineStr">
         <is>
           <t>Richard Rowe (Director Chief Executive Officer)</t>
@@ -11518,7 +11606,11 @@
           <t>Director, Information Technology Operations &amp; Infrastru...</t>
         </is>
       </c>
-      <c r="M108" s="2" t="n"/>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>pjoy@healthcaresouth.com</t>
+        </is>
+      </c>
       <c r="N108" s="2" t="n"/>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -11624,7 +11716,11 @@
           <t>Senior Software Systems Engineer &amp; Director &amp; Electrica...</t>
         </is>
       </c>
-      <c r="M109" s="4" t="n"/>
+      <c r="M109" s="4" t="inlineStr">
+        <is>
+          <t>jgh@massa.com</t>
+        </is>
+      </c>
       <c r="N109" s="4" t="inlineStr">
         <is>
           <t>Donald Massa (Chief Technical Officer &amp; Chairman)</t>
@@ -11734,7 +11830,11 @@
           <t>Vice President, Chief Information Officer</t>
         </is>
       </c>
-      <c r="M110" s="4" t="n"/>
+      <c r="M110" s="4" t="inlineStr">
+        <is>
+          <t>danielbagley@hinghamsavings.com</t>
+        </is>
+      </c>
       <c r="N110" s="4" t="inlineStr">
         <is>
           <t>Patrick Gaughen (President &amp; Chief Operating Officer)</t>
@@ -13354,7 +13454,11 @@
           <t>Director, Information Technology &amp; Development</t>
         </is>
       </c>
-      <c r="M126" s="4" t="n"/>
+      <c r="M126" s="4" t="inlineStr">
+        <is>
+          <t>pmurphy@bsm.com</t>
+        </is>
+      </c>
       <c r="N126" s="4" t="inlineStr">
         <is>
           <t>Alain Hanna (Chief Financial Officer)</t>
@@ -13468,7 +13572,11 @@
           <t>Chief Information Officer</t>
         </is>
       </c>
-      <c r="M127" s="2" t="n"/>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>shawk@manetchc.org</t>
+        </is>
+      </c>
       <c r="N127" s="2" t="inlineStr">
         <is>
           <t>Marc Conroy (Chief Financial Officer)</t>
@@ -13692,7 +13800,11 @@
           <t>Chief Information Officer</t>
         </is>
       </c>
-      <c r="M129" s="2" t="n"/>
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>jbrudnick@xsbrokers.com</t>
+        </is>
+      </c>
       <c r="N129" s="2" t="inlineStr">
         <is>
           <t>Eric Wirkus (Chief Executive Officer)</t>
@@ -15348,7 +15460,11 @@
           <t>Chief Information Officer</t>
         </is>
       </c>
-      <c r="M145" s="4" t="n"/>
+      <c r="M145" s="4" t="inlineStr">
+        <is>
+          <t>aivkovic@cdf1.com</t>
+        </is>
+      </c>
       <c r="N145" s="4" t="inlineStr">
         <is>
           <t>Joseph Sullivan (President)</t>
@@ -15760,7 +15876,11 @@
           <t>Systems Technician</t>
         </is>
       </c>
-      <c r="M149" s="2" t="n"/>
+      <c r="M149" s="2" t="inlineStr">
+        <is>
+          <t>tstevenson@vptec.com</t>
+        </is>
+      </c>
       <c r="N149" s="2" t="n"/>
       <c r="O149" s="2" t="inlineStr">
         <is>
@@ -15866,7 +15986,11 @@
       </c>
       <c r="K150" s="2" t="n"/>
       <c r="L150" s="2" t="n"/>
-      <c r="M150" s="2" t="n"/>
+      <c r="M150" s="2" t="inlineStr">
+        <is>
+          <t>soliver@pbortho.com</t>
+        </is>
+      </c>
       <c r="N150" s="2" t="inlineStr">
         <is>
           <t>Scott Oliver (President &amp; Founder)</t>
@@ -17196,7 +17320,11 @@
           <t>IT Support Technician</t>
         </is>
       </c>
-      <c r="M163" s="4" t="n"/>
+      <c r="M163" s="4" t="inlineStr">
+        <is>
+          <t>w.arensman@ee-co.com</t>
+        </is>
+      </c>
       <c r="N163" s="4" t="inlineStr">
         <is>
           <t>Kyle Willis (President &amp; Chief Operating Officer)</t>
@@ -17538,7 +17666,11 @@
           <t>IT Specialist</t>
         </is>
       </c>
-      <c r="M166" s="4" t="n"/>
+      <c r="M166" s="4" t="inlineStr">
+        <is>
+          <t>lgray@rexa.com</t>
+        </is>
+      </c>
       <c r="N166" s="4" t="n"/>
       <c r="O166" s="4" t="inlineStr">
         <is>
@@ -17644,7 +17776,11 @@
           <t>Manager, Management Information Systems</t>
         </is>
       </c>
-      <c r="M167" s="4" t="n"/>
+      <c r="M167" s="4" t="inlineStr">
+        <is>
+          <t>mbadilla@pharmasol.com</t>
+        </is>
+      </c>
       <c r="N167" s="4" t="inlineStr">
         <is>
           <t>Donghwan Choi (President)</t>
@@ -17758,7 +17894,11 @@
           <t>Senior VP, Information Security</t>
         </is>
       </c>
-      <c r="M168" s="2" t="n"/>
+      <c r="M168" s="2" t="inlineStr">
+        <is>
+          <t>ppijanowski@scucu.com</t>
+        </is>
+      </c>
       <c r="N168" s="2" t="inlineStr">
         <is>
           <t>Robert Gustafson (President &amp; Chief Executive Officer)</t>
@@ -17864,7 +18004,11 @@
       </c>
       <c r="K169" s="2" t="n"/>
       <c r="L169" s="2" t="n"/>
-      <c r="M169" s="2" t="n"/>
+      <c r="M169" s="2" t="inlineStr">
+        <is>
+          <t>starallo@lyne.com</t>
+        </is>
+      </c>
       <c r="N169" s="2" t="inlineStr">
         <is>
           <t>Stephen Tarallo (President &amp; Chief Executive Officer &amp; Director)</t>
@@ -19876,7 +20020,11 @@
           <t>CISO &amp; Director, Infrastructure</t>
         </is>
       </c>
-      <c r="M189" s="2" t="n"/>
+      <c r="M189" s="2" t="inlineStr">
+        <is>
+          <t>tom_kane@bostonmutual.com</t>
+        </is>
+      </c>
       <c r="N189" s="2" t="n"/>
       <c r="O189" s="2" t="inlineStr">
         <is>
@@ -20530,7 +20678,11 @@
           <t>Business &amp; IT Systems Analyst</t>
         </is>
       </c>
-      <c r="M196" s="2" t="n"/>
+      <c r="M196" s="2" t="inlineStr">
+        <is>
+          <t>rkouatcho@lacerta.com</t>
+        </is>
+      </c>
       <c r="N196" s="2" t="inlineStr">
         <is>
           <t>Ali Lotfi (President)</t>
@@ -20644,7 +20796,11 @@
           <t>Manager, Information Technology</t>
         </is>
       </c>
-      <c r="M197" s="2" t="n"/>
+      <c r="M197" s="2" t="inlineStr">
+        <is>
+          <t>bgabriel@metalbellows.com</t>
+        </is>
+      </c>
       <c r="N197" s="2" t="n"/>
       <c r="O197" s="2" t="inlineStr">
         <is>
@@ -20970,7 +21126,11 @@
       </c>
       <c r="K200" s="2" t="n"/>
       <c r="L200" s="2" t="n"/>
-      <c r="M200" s="2" t="n"/>
+      <c r="M200" s="2" t="inlineStr">
+        <is>
+          <t>tony@proven-process.com</t>
+        </is>
+      </c>
       <c r="N200" s="2" t="inlineStr">
         <is>
           <t>Anthony Roscoe (Business Owner)</t>
@@ -21088,7 +21248,11 @@
           <t>Vice President, Compliance &amp; Business Systems</t>
         </is>
       </c>
-      <c r="M201" s="2" t="n"/>
+      <c r="M201" s="2" t="inlineStr">
+        <is>
+          <t>dking@acumentrics.com</t>
+        </is>
+      </c>
       <c r="N201" s="2" t="inlineStr">
         <is>
           <t>John Cerulli (Chief Executive Officer)</t>
@@ -21194,7 +21358,11 @@
       </c>
       <c r="K202" s="2" t="n"/>
       <c r="L202" s="2" t="n"/>
-      <c r="M202" s="2" t="n"/>
+      <c r="M202" s="2" t="inlineStr">
+        <is>
+          <t>lonnie@clinicalsciencelab.com</t>
+        </is>
+      </c>
       <c r="N202" s="2" t="inlineStr">
         <is>
           <t>Lonnie Elfbaum (Chief Financial Officer &amp; Controller)</t>
@@ -43807,7 +43975,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>ccastellano@cutterassociates.com</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -44216,7 +44388,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>mfederico@rfcu.com</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -44275,7 +44451,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>darrell@uppababy.com</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -44393,7 +44573,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>sskorohod@briggsengineering.com</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
@@ -45128,7 +45312,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G25" s="2" t="n"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>jamesc@zildjian.com</t>
+        </is>
+      </c>
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="2" t="inlineStr">
         <is>
@@ -45246,7 +45434,11 @@
           <t>Company main line -- reliably sourced</t>
         </is>
       </c>
-      <c r="G27" s="2" t="n"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>slutz@nvna.org</t>
+        </is>
+      </c>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="2" t="inlineStr">
         <is>
@@ -45364,7 +45556,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>wayne@miniter.com</t>
+        </is>
+      </c>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="2" t="inlineStr">
         <is>
@@ -45423,7 +45619,11 @@
           <t>Company main line -- reliably sourced</t>
         </is>
       </c>
-      <c r="G30" s="2" t="n"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>danielle.jones@snowandjones.com</t>
+        </is>
+      </c>
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="2" t="inlineStr">
         <is>
@@ -45482,7 +45682,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G31" s="2" t="n"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>randallsteele@airxchange.com</t>
+        </is>
+      </c>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="inlineStr">
         <is>
@@ -46677,7 +46881,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G52" s="2" t="n"/>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>emoniz@cushingcenters.org</t>
+        </is>
+      </c>
       <c r="H52" s="2" t="n"/>
       <c r="I52" s="2" t="inlineStr">
         <is>
@@ -47141,7 +47349,11 @@
           <t>Company main line -- reliably sourced</t>
         </is>
       </c>
-      <c r="G60" s="2" t="n"/>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>aemma@palanders.com</t>
+        </is>
+      </c>
       <c r="H60" s="2" t="n"/>
       <c r="I60" s="2" t="inlineStr">
         <is>
@@ -47200,7 +47412,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G61" s="2" t="n"/>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>dmelo@buckleyonline.com</t>
+        </is>
+      </c>
       <c r="H61" s="2" t="n"/>
       <c r="I61" s="2" t="inlineStr">
         <is>
@@ -47259,7 +47475,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G62" s="2" t="n"/>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>lraasch@srcmedical.com</t>
+        </is>
+      </c>
       <c r="H62" s="2" t="n"/>
       <c r="I62" s="2" t="inlineStr">
         <is>
@@ -47318,7 +47538,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G63" s="2" t="n"/>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>daniel_mcclelland@hapcoincorporated.com</t>
+        </is>
+      </c>
       <c r="H63" s="2" t="n"/>
       <c r="I63" s="2" t="inlineStr">
         <is>
@@ -47377,7 +47601,11 @@
           <t>Company main line -- reliably sourced</t>
         </is>
       </c>
-      <c r="G64" s="2" t="n"/>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>mphung@gemgravure.com</t>
+        </is>
+      </c>
       <c r="H64" s="2" t="n"/>
       <c r="I64" s="2" t="inlineStr">
         <is>
@@ -47880,7 +48108,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G73" s="2" t="n"/>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>jnoel@royalhealthgroup.com</t>
+        </is>
+      </c>
       <c r="H73" s="2" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
@@ -47994,7 +48226,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G75" s="2" t="n"/>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>cgeer@thayerscale.com</t>
+        </is>
+      </c>
       <c r="H75" s="2" t="n"/>
       <c r="I75" s="2" t="inlineStr">
         <is>
@@ -48953,7 +49189,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G92" s="2" t="n"/>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>pcleary@tkasphalt.com</t>
+        </is>
+      </c>
       <c r="H92" s="2" t="n"/>
       <c r="I92" s="2" t="inlineStr">
         <is>
@@ -49012,7 +49252,11 @@
           <t>Company main line -- reliably sourced</t>
         </is>
       </c>
-      <c r="G93" s="2" t="n"/>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>tmcmanus@cclco.com</t>
+        </is>
+      </c>
       <c r="H93" s="2" t="n"/>
       <c r="I93" s="2" t="inlineStr">
         <is>
@@ -49688,7 +49932,11 @@
           <t>Company main line -- reliably sourced</t>
         </is>
       </c>
-      <c r="G105" s="2" t="n"/>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>ltempesta@southshorebank.com</t>
+        </is>
+      </c>
       <c r="H105" s="2" t="n"/>
       <c r="I105" s="2" t="inlineStr">
         <is>
@@ -49747,7 +49995,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G106" s="2" t="n"/>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>kroche@electroswitch.com</t>
+        </is>
+      </c>
       <c r="H106" s="2" t="n"/>
       <c r="I106" s="2" t="inlineStr">
         <is>
@@ -49806,7 +50058,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G107" s="2" t="n"/>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>mruuska@coastalheritagebank.com</t>
+        </is>
+      </c>
       <c r="H107" s="2" t="n"/>
       <c r="I107" s="2" t="inlineStr">
         <is>
@@ -49865,7 +50121,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G108" s="2" t="n"/>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>pjoy@healthcaresouth.com</t>
+        </is>
+      </c>
       <c r="H108" s="2" t="n"/>
       <c r="I108" s="2" t="inlineStr">
         <is>
@@ -49924,7 +50184,11 @@
           <t>Company main line -- reliably sourced</t>
         </is>
       </c>
-      <c r="G109" s="2" t="n"/>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>jgh@massa.com</t>
+        </is>
+      </c>
       <c r="H109" s="2" t="n"/>
       <c r="I109" s="2" t="inlineStr">
         <is>
@@ -49983,7 +50247,11 @@
           <t>Company main line -- reliably sourced</t>
         </is>
       </c>
-      <c r="G110" s="2" t="n"/>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>danielbagley@hinghamsavings.com</t>
+        </is>
+      </c>
       <c r="H110" s="2" t="n"/>
       <c r="I110" s="2" t="inlineStr">
         <is>
@@ -50895,7 +51163,11 @@
           <t>Company main line -- reliably sourced</t>
         </is>
       </c>
-      <c r="G126" s="2" t="n"/>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>pmurphy@bsm.com</t>
+        </is>
+      </c>
       <c r="H126" s="2" t="n"/>
       <c r="I126" s="2" t="inlineStr">
         <is>
@@ -50954,7 +51226,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G127" s="2" t="n"/>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>shawk@manetchc.org</t>
+        </is>
+      </c>
       <c r="H127" s="2" t="n"/>
       <c r="I127" s="2" t="inlineStr">
         <is>
@@ -51072,7 +51348,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G129" s="2" t="n"/>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>jbrudnick@xsbrokers.com</t>
+        </is>
+      </c>
       <c r="H129" s="2" t="n"/>
       <c r="I129" s="2" t="inlineStr">
         <is>
@@ -51988,7 +52268,11 @@
           <t>Company main line -- reliably sourced</t>
         </is>
       </c>
-      <c r="G145" s="2" t="n"/>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>aivkovic@cdf1.com</t>
+        </is>
+      </c>
       <c r="H145" s="2" t="n"/>
       <c r="I145" s="2" t="inlineStr">
         <is>
@@ -52216,7 +52500,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G149" s="2" t="n"/>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>tstevenson@vptec.com</t>
+        </is>
+      </c>
       <c r="H149" s="2" t="n"/>
       <c r="I149" s="2" t="inlineStr">
         <is>
@@ -52275,7 +52563,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G150" s="2" t="n"/>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>soliver@pbortho.com</t>
+        </is>
+      </c>
       <c r="H150" s="2" t="n"/>
       <c r="I150" s="2" t="inlineStr">
         <is>
@@ -53010,7 +53302,11 @@
           <t>Company main line -- reliably sourced</t>
         </is>
       </c>
-      <c r="G163" s="2" t="n"/>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>w.arensman@ee-co.com</t>
+        </is>
+      </c>
       <c r="H163" s="2" t="n"/>
       <c r="I163" s="2" t="inlineStr">
         <is>
@@ -53187,7 +53483,11 @@
           <t>Company main line -- reliably sourced</t>
         </is>
       </c>
-      <c r="G166" s="2" t="n"/>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>lgray@rexa.com</t>
+        </is>
+      </c>
       <c r="H166" s="2" t="n"/>
       <c r="I166" s="2" t="inlineStr">
         <is>
@@ -53246,7 +53546,11 @@
           <t>Company main line -- reliably sourced</t>
         </is>
       </c>
-      <c r="G167" s="2" t="n"/>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>mbadilla@pharmasol.com</t>
+        </is>
+      </c>
       <c r="H167" s="2" t="n"/>
       <c r="I167" s="2" t="inlineStr">
         <is>
@@ -53305,7 +53609,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G168" s="2" t="n"/>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>ppijanowski@scucu.com</t>
+        </is>
+      </c>
       <c r="H168" s="2" t="n"/>
       <c r="I168" s="2" t="inlineStr">
         <is>
@@ -53364,7 +53672,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G169" s="2" t="n"/>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>starallo@lyne.com</t>
+        </is>
+      </c>
       <c r="H169" s="2" t="n"/>
       <c r="I169" s="2" t="inlineStr">
         <is>
@@ -54382,7 +54694,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G187" s="2" t="n"/>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>tom_kane@bostonmutual.com</t>
+        </is>
+      </c>
       <c r="H187" s="2" t="n"/>
       <c r="I187" s="2" t="inlineStr">
         <is>
@@ -54724,7 +55040,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G193" s="2" t="n"/>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t>rkouatcho@lacerta.com</t>
+        </is>
+      </c>
       <c r="H193" s="2" t="n"/>
       <c r="I193" s="2" t="inlineStr">
         <is>
@@ -54783,7 +55103,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G194" s="2" t="n"/>
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t>bgabriel@metalbellows.com</t>
+        </is>
+      </c>
       <c r="H194" s="2" t="n"/>
       <c r="I194" s="2" t="inlineStr">
         <is>
@@ -54960,7 +55284,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G197" s="2" t="n"/>
+      <c r="G197" s="2" t="inlineStr">
+        <is>
+          <t>tony@proven-process.com</t>
+        </is>
+      </c>
       <c r="H197" s="2" t="n"/>
       <c r="I197" s="2" t="inlineStr">
         <is>
@@ -55019,7 +55347,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G198" s="2" t="n"/>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>dking@acumentrics.com</t>
+        </is>
+      </c>
       <c r="H198" s="2" t="n"/>
       <c r="I198" s="2" t="inlineStr">
         <is>
@@ -55078,7 +55410,11 @@
           <t>ZoomInfo verified personal direct/mobile</t>
         </is>
       </c>
-      <c r="G199" s="2" t="n"/>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t>lonnie@clinicalsciencelab.com</t>
+        </is>
+      </c>
       <c r="H199" s="2" t="n"/>
       <c r="I199" s="2" t="inlineStr">
         <is>

</xml_diff>